<commit_message>
added lfs to track videos
</commit_message>
<xml_diff>
--- a/data/status_report.xlsx
+++ b/data/status_report.xlsx
@@ -1408,7 +1408,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>71.67700000000001</v>
+        <v>63.88</v>
       </c>
       <c r="F10" t="n">
         <v>-82.26600000000001</v>
@@ -1419,20 +1419,20 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1.45</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>1.12</v>
+        <v>0.52</v>
       </c>
       <c r="J10" t="n">
-        <v>1.45</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K10" t="n">
         <v>2681</v>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>21 runs (top 5 by duration): f455–f459 (7.6s–7.7s, 0.1s) | f85–f88 (1.4s–1.5s, 0.1s) | f222–f224 (3.7s–3.7s, 0.0s) | f259–f260 (4.3s–4.3s, 0.0s) | f523–f524 (8.7s–8.7s, 0.0s) ... and 16 more</t>
+          <t>7 runs: f85–f88 (1.4s–1.5s, 0.1s) | f163 (2.7s, isolated) | f223–f224 (3.7s–3.7s, 0.0s) | f259–f260 (4.3s–4.3s, 0.0s) | f419–f420 (7.0s–7.0s, 0.0s) | f561–f562 (9.4s–9.4s, 0.0s) | f666–f667 (11.1s–11.1s, 0.0s)</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -1715,10 +1715,10 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>1 run: f97–f98 (1.6s–1.6s, 0.0s)</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -1786,27 +1786,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>th1_p093_th2_m002</t>
+          <t>th1_p092_th2_m002</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DSC_0156</t>
+          <t>DSC_0161</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>th1_p093_th2_m002.mov</t>
+          <t>th1_p092_th2_m002.mov</t>
         </is>
       </c>
       <c r="D14" t="n">
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>90</v>
+        <v>81.968</v>
       </c>
       <c r="F14" t="n">
-        <v>-2.148</v>
+        <v>-1.757</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1814,20 +1814,20 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>2599</v>
+        <v>2453</v>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>1 isolated frame</t>
+          <t>none</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -1880,27 +1880,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>th1_p093_th2_m000</t>
+          <t>th1_p090_th2_p000</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DSC_0157</t>
+          <t>DSC_0160</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>th1_p093_th2_m000.mov</t>
+          <t>th1_p090_th2_p000.mov</t>
         </is>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>90</v>
+        <v>82.26600000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.768</v>
+        <v>1.768</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1908,20 +1908,20 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>2037</v>
+        <v>88</v>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>1 run: f102–f104 (1.7s–1.7s, 0.0s)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>per-video</t>
+          <t>global</t>
         </is>
       </c>
       <c r="V15" s="3" t="inlineStr"/>
@@ -1974,48 +1974,48 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>th1_p091_th2_m001</t>
+          <t>th1_p093_th2_m002</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DSC_0162</t>
+          <t>DSC_0156</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>th1_p091_th2_m001.mov</t>
+          <t>th1_p093_th2_m002.mov</t>
         </is>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>90.354</v>
+        <v>90</v>
       </c>
       <c r="F16" t="n">
-        <v>-1.406</v>
+        <v>-2.148</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>TRACKED — analysis pending</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>5.77</v>
+      <c r="H16" t="n">
+        <v>0.04</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>5.77</v>
+        <v>0.04</v>
       </c>
       <c r="K16" t="n">
-        <v>1958</v>
+        <v>2599</v>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>10 runs: f115 (1.9s, isolated) | f146–f147 (2.4s–2.5s, 0.0s) | f157–f161 (2.6s–2.7s, 0.1s) | f163 (2.7s, isolated) | f165–f166 (2.8s–2.8s, 0.0s) | f196 (3.3s, isolated) | f198–f250 (3.3s–4.2s, 0.9s) | f252–f291 (4.2s–4.9s, 0.7s) | f293–f299 (4.9s–5.0s, 0.1s) | f301 (5.0s, isolated)</t>
+          <t>1 isolated frame</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -2063,36 +2063,32 @@
           <t>per-video</t>
         </is>
       </c>
-      <c r="V16" s="3" t="inlineStr">
-        <is>
-          <t>verification: DOWNGRADED via chaos audit on 2026-05-02: was 'verified'; new verdict WARN. Reasons: free-swing dropout 5.8% in 5–10% band; 62 residual suspects post-interpolation; 62 arm-length violation(s) (max deviation 33.1%) — tracker latched on wrong object; 62 frame(s) with |Δω| spike (unphysical acceleration)</t>
-        </is>
-      </c>
+      <c r="V16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>th1_p092_th2_m002</t>
+          <t>th1_p093_th2_m000</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DSC_0161</t>
+          <t>DSC_0157</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>th1_p092_th2_m002.mov</t>
+          <t>th1_p093_th2_m000.mov</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>90.703</v>
+        <v>90</v>
       </c>
       <c r="F17" t="n">
-        <v>-2.108</v>
+        <v>-1.768</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -2100,20 +2096,20 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="K17" t="n">
-        <v>2453</v>
+        <v>2037</v>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>1 run: f102–f104 (1.7s–1.7s, 0.0s)</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -2166,48 +2162,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>th1_p090_th2_p000</t>
+          <t>th1_p091_th2_m001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DSC_0160</t>
+          <t>DSC_0162</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>th1_p090_th2_p000.mov</t>
+          <t>th1_p091_th2_m001.mov</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>91.06100000000001</v>
+        <v>90.354</v>
       </c>
       <c r="F18" t="n">
-        <v>1.414</v>
+        <v>-1.406</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>TRACKED — analysis pending</t>
         </is>
       </c>
-      <c r="H18" t="n">
-        <v>0</v>
+      <c r="H18" s="2" t="n">
+        <v>5.77</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>5.77</v>
       </c>
       <c r="K18" t="n">
-        <v>88</v>
+        <v>1958</v>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>10 runs: f115 (1.9s, isolated) | f146–f147 (2.4s–2.5s, 0.0s) | f157–f161 (2.6s–2.7s, 0.1s) | f163 (2.7s, isolated) | f165–f166 (2.8s–2.8s, 0.0s) | f196 (3.3s, isolated) | f198–f250 (3.3s–4.2s, 0.9s) | f252–f291 (4.2s–4.9s, 0.7s) | f293–f299 (4.9s–5.0s, 0.1s) | f301 (5.0s, isolated)</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -2252,10 +2248,14 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>global</t>
-        </is>
-      </c>
-      <c r="V18" s="3" t="inlineStr"/>
+          <t>per-video</t>
+        </is>
+      </c>
+      <c r="V18" s="3" t="inlineStr">
+        <is>
+          <t>verification: DOWNGRADED via chaos audit on 2026-05-02: was 'verified'; new verdict WARN. Reasons: free-swing dropout 5.8% in 5–10% band; 62 residual suspects post-interpolation; 62 arm-length violation(s) (max deviation 33.1%) — tracker latched on wrong object; 62 frame(s) with |Δω| spike (unphysical acceleration)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">

</xml_diff>